<commit_message>
feat(portfolio): ativar Lay Away Fortaleza 1X (Fav<=1.40 | O25>=1.75) nas Paginas 01, 02 e automacao
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-09-03.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-09-03.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,6 +529,21 @@
           <t>PnL_R$</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Lucro_Green_R$</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -615,6 +630,9 @@
       <c r="T2" t="n">
         <v>19.39</v>
       </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -700,6 +718,88 @@
       </c>
       <c r="T3" t="n">
         <v>16.97</v>
+      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>COLOMBIA 1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>America De Cali x Alianza</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Lay Away Fortaleza 1X (Fav &lt;= 1.40 | O25 &gt;= 1.75)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Match Odds (Away)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="L4" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="M4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>3x0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="V4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>LIQUIDADO</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>